<commit_message>
Ajout des exemples CDA pour validation (#42)
* test examples

* update

* resolve bugs

* test

* rm ext

* text example

* text example

* text example

* add more examples

* rename

* update

* update

* add working exam

* update examples

* update

* update edisp med

* update

* update edisp med

* add ips

* update termino 7ee806c3791576358559f28b96bb563eafdc00bc
</commit_message>
<xml_diff>
--- a/main/ig/StructureDefinition-fr-practitioner-document.xlsx
+++ b/main/ig/StructureDefinition-fr-practitioner-document.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13901" uniqueCount="1008">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13902" uniqueCount="1007">
   <si>
     <t>Property</t>
   </si>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-08-01T08:11:50+00:00</t>
+    <t>2025-08-22T10:16:53+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -2869,9 +2869,6 @@
   </si>
   <si>
     <t>Practitioner.qualification:savoirFaire/professionMedecin.code.coding:savoirFaire</t>
-  </si>
-  <si>
-    <t>https://interop.esante.gouv.fr/ig/document/core/ValueSet/fr-doc-vs-savoir-faire-profession-medecin</t>
   </si>
   <si>
     <t>Practitioner.qualification:savoirFaire/professionMedecin.code.coding:typeSavoirFaire</t>
@@ -39063,11 +39060,13 @@
         <v>84</v>
       </c>
       <c r="X265" t="s" s="2">
-        <v>249</v>
-      </c>
-      <c r="Y265" s="2"/>
+        <v>84</v>
+      </c>
+      <c r="Y265" t="s" s="2">
+        <v>84</v>
+      </c>
       <c r="Z265" t="s" s="2">
-        <v>923</v>
+        <v>84</v>
       </c>
       <c r="AA265" t="s" s="2">
         <v>84</v>
@@ -39135,7 +39134,7 @@
     </row>
     <row r="266" hidden="true">
       <c r="A266" t="s" s="2">
-        <v>924</v>
+        <v>923</v>
       </c>
       <c r="B266" t="s" s="2">
         <v>809</v>
@@ -39204,7 +39203,7 @@
       </c>
       <c r="Y266" s="2"/>
       <c r="Z266" t="s" s="2">
-        <v>925</v>
+        <v>924</v>
       </c>
       <c r="AA266" t="s" s="2">
         <v>84</v>
@@ -39272,7 +39271,7 @@
     </row>
     <row r="267" hidden="true">
       <c r="A267" t="s" s="2">
-        <v>926</v>
+        <v>925</v>
       </c>
       <c r="B267" t="s" s="2">
         <v>824</v>
@@ -39409,7 +39408,7 @@
     </row>
     <row r="268" hidden="true">
       <c r="A268" t="s" s="2">
-        <v>927</v>
+        <v>926</v>
       </c>
       <c r="B268" t="s" s="2">
         <v>743</v>
@@ -39544,7 +39543,7 @@
     </row>
     <row r="269" hidden="true">
       <c r="A269" t="s" s="2">
-        <v>928</v>
+        <v>927</v>
       </c>
       <c r="B269" t="s" s="2">
         <v>749</v>
@@ -39677,13 +39676,13 @@
     </row>
     <row r="270" hidden="true">
       <c r="A270" t="s" s="2">
-        <v>929</v>
+        <v>928</v>
       </c>
       <c r="B270" t="s" s="2">
         <v>715</v>
       </c>
       <c r="C270" t="s" s="2">
-        <v>930</v>
+        <v>929</v>
       </c>
       <c r="D270" t="s" s="2">
         <v>84</v>
@@ -39708,7 +39707,7 @@
         <v>716</v>
       </c>
       <c r="L270" t="s" s="2">
-        <v>931</v>
+        <v>930</v>
       </c>
       <c r="M270" t="s" s="2">
         <v>718</v>
@@ -39812,7 +39811,7 @@
     </row>
     <row r="271" hidden="true">
       <c r="A271" t="s" s="2">
-        <v>932</v>
+        <v>931</v>
       </c>
       <c r="B271" t="s" s="2">
         <v>723</v>
@@ -39945,7 +39944,7 @@
     </row>
     <row r="272" hidden="true">
       <c r="A272" t="s" s="2">
-        <v>933</v>
+        <v>932</v>
       </c>
       <c r="B272" t="s" s="2">
         <v>724</v>
@@ -40080,7 +40079,7 @@
     </row>
     <row r="273" hidden="true">
       <c r="A273" t="s" s="2">
-        <v>934</v>
+        <v>933</v>
       </c>
       <c r="B273" t="s" s="2">
         <v>725</v>
@@ -40217,7 +40216,7 @@
     </row>
     <row r="274" hidden="true">
       <c r="A274" t="s" s="2">
-        <v>935</v>
+        <v>934</v>
       </c>
       <c r="B274" t="s" s="2">
         <v>730</v>
@@ -40352,7 +40351,7 @@
     </row>
     <row r="275" hidden="true">
       <c r="A275" t="s" s="2">
-        <v>936</v>
+        <v>935</v>
       </c>
       <c r="B275" t="s" s="2">
         <v>736</v>
@@ -40485,7 +40484,7 @@
     </row>
     <row r="276" hidden="true">
       <c r="A276" t="s" s="2">
-        <v>937</v>
+        <v>936</v>
       </c>
       <c r="B276" t="s" s="2">
         <v>805</v>
@@ -40618,7 +40617,7 @@
     </row>
     <row r="277" hidden="true">
       <c r="A277" t="s" s="2">
-        <v>938</v>
+        <v>937</v>
       </c>
       <c r="B277" t="s" s="2">
         <v>807</v>
@@ -40753,7 +40752,7 @@
     </row>
     <row r="278" hidden="true">
       <c r="A278" t="s" s="2">
-        <v>939</v>
+        <v>938</v>
       </c>
       <c r="B278" t="s" s="2">
         <v>809</v>
@@ -40888,7 +40887,7 @@
     </row>
     <row r="279" hidden="true">
       <c r="A279" t="s" s="2">
-        <v>940</v>
+        <v>939</v>
       </c>
       <c r="B279" t="s" s="2">
         <v>809</v>
@@ -40957,7 +40956,7 @@
       </c>
       <c r="Y279" s="2"/>
       <c r="Z279" t="s" s="2">
-        <v>941</v>
+        <v>940</v>
       </c>
       <c r="AA279" t="s" s="2">
         <v>84</v>
@@ -41025,7 +41024,7 @@
     </row>
     <row r="280" hidden="true">
       <c r="A280" t="s" s="2">
-        <v>942</v>
+        <v>941</v>
       </c>
       <c r="B280" t="s" s="2">
         <v>809</v>
@@ -41094,7 +41093,7 @@
       </c>
       <c r="Y280" s="2"/>
       <c r="Z280" t="s" s="2">
-        <v>943</v>
+        <v>942</v>
       </c>
       <c r="AA280" t="s" s="2">
         <v>84</v>
@@ -41162,7 +41161,7 @@
     </row>
     <row r="281" hidden="true">
       <c r="A281" t="s" s="2">
-        <v>944</v>
+        <v>943</v>
       </c>
       <c r="B281" t="s" s="2">
         <v>824</v>
@@ -41299,7 +41298,7 @@
     </row>
     <row r="282" hidden="true">
       <c r="A282" t="s" s="2">
-        <v>945</v>
+        <v>944</v>
       </c>
       <c r="B282" t="s" s="2">
         <v>743</v>
@@ -41434,7 +41433,7 @@
     </row>
     <row r="283" hidden="true">
       <c r="A283" t="s" s="2">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="B283" t="s" s="2">
         <v>749</v>
@@ -41567,13 +41566,13 @@
     </row>
     <row r="284" hidden="true">
       <c r="A284" t="s" s="2">
-        <v>947</v>
+        <v>946</v>
       </c>
       <c r="B284" t="s" s="2">
         <v>715</v>
       </c>
       <c r="C284" t="s" s="2">
-        <v>948</v>
+        <v>947</v>
       </c>
       <c r="D284" t="s" s="2">
         <v>84</v>
@@ -41598,7 +41597,7 @@
         <v>716</v>
       </c>
       <c r="L284" t="s" s="2">
-        <v>949</v>
+        <v>948</v>
       </c>
       <c r="M284" t="s" s="2">
         <v>718</v>
@@ -41702,7 +41701,7 @@
     </row>
     <row r="285" hidden="true">
       <c r="A285" t="s" s="2">
-        <v>950</v>
+        <v>949</v>
       </c>
       <c r="B285" t="s" s="2">
         <v>723</v>
@@ -41835,7 +41834,7 @@
     </row>
     <row r="286" hidden="true">
       <c r="A286" t="s" s="2">
-        <v>951</v>
+        <v>950</v>
       </c>
       <c r="B286" t="s" s="2">
         <v>724</v>
@@ -41970,7 +41969,7 @@
     </row>
     <row r="287" hidden="true">
       <c r="A287" t="s" s="2">
-        <v>952</v>
+        <v>951</v>
       </c>
       <c r="B287" t="s" s="2">
         <v>725</v>
@@ -42107,7 +42106,7 @@
     </row>
     <row r="288" hidden="true">
       <c r="A288" t="s" s="2">
-        <v>953</v>
+        <v>952</v>
       </c>
       <c r="B288" t="s" s="2">
         <v>730</v>
@@ -42242,7 +42241,7 @@
     </row>
     <row r="289" hidden="true">
       <c r="A289" t="s" s="2">
-        <v>954</v>
+        <v>953</v>
       </c>
       <c r="B289" t="s" s="2">
         <v>736</v>
@@ -42375,7 +42374,7 @@
     </row>
     <row r="290" hidden="true">
       <c r="A290" t="s" s="2">
-        <v>955</v>
+        <v>954</v>
       </c>
       <c r="B290" t="s" s="2">
         <v>805</v>
@@ -42508,7 +42507,7 @@
     </row>
     <row r="291" hidden="true">
       <c r="A291" t="s" s="2">
-        <v>956</v>
+        <v>955</v>
       </c>
       <c r="B291" t="s" s="2">
         <v>807</v>
@@ -42643,7 +42642,7 @@
     </row>
     <row r="292" hidden="true">
       <c r="A292" t="s" s="2">
-        <v>957</v>
+        <v>956</v>
       </c>
       <c r="B292" t="s" s="2">
         <v>809</v>
@@ -42778,7 +42777,7 @@
     </row>
     <row r="293" hidden="true">
       <c r="A293" t="s" s="2">
-        <v>958</v>
+        <v>957</v>
       </c>
       <c r="B293" t="s" s="2">
         <v>809</v>
@@ -42847,7 +42846,7 @@
       </c>
       <c r="Y293" s="2"/>
       <c r="Z293" t="s" s="2">
-        <v>959</v>
+        <v>958</v>
       </c>
       <c r="AA293" t="s" s="2">
         <v>84</v>
@@ -42915,7 +42914,7 @@
     </row>
     <row r="294" hidden="true">
       <c r="A294" t="s" s="2">
-        <v>960</v>
+        <v>959</v>
       </c>
       <c r="B294" t="s" s="2">
         <v>809</v>
@@ -42984,7 +42983,7 @@
       </c>
       <c r="Y294" s="2"/>
       <c r="Z294" t="s" s="2">
-        <v>961</v>
+        <v>960</v>
       </c>
       <c r="AA294" t="s" s="2">
         <v>84</v>
@@ -43052,7 +43051,7 @@
     </row>
     <row r="295" hidden="true">
       <c r="A295" t="s" s="2">
-        <v>962</v>
+        <v>961</v>
       </c>
       <c r="B295" t="s" s="2">
         <v>824</v>
@@ -43189,7 +43188,7 @@
     </row>
     <row r="296" hidden="true">
       <c r="A296" t="s" s="2">
-        <v>963</v>
+        <v>962</v>
       </c>
       <c r="B296" t="s" s="2">
         <v>743</v>
@@ -43324,7 +43323,7 @@
     </row>
     <row r="297" hidden="true">
       <c r="A297" t="s" s="2">
-        <v>964</v>
+        <v>963</v>
       </c>
       <c r="B297" t="s" s="2">
         <v>749</v>
@@ -43457,13 +43456,13 @@
     </row>
     <row r="298" hidden="true">
       <c r="A298" t="s" s="2">
-        <v>965</v>
+        <v>964</v>
       </c>
       <c r="B298" t="s" s="2">
         <v>715</v>
       </c>
       <c r="C298" t="s" s="2">
-        <v>966</v>
+        <v>965</v>
       </c>
       <c r="D298" t="s" s="2">
         <v>84</v>
@@ -43488,7 +43487,7 @@
         <v>716</v>
       </c>
       <c r="L298" t="s" s="2">
-        <v>967</v>
+        <v>966</v>
       </c>
       <c r="M298" t="s" s="2">
         <v>718</v>
@@ -43592,7 +43591,7 @@
     </row>
     <row r="299" hidden="true">
       <c r="A299" t="s" s="2">
-        <v>968</v>
+        <v>967</v>
       </c>
       <c r="B299" t="s" s="2">
         <v>723</v>
@@ -43725,7 +43724,7 @@
     </row>
     <row r="300" hidden="true">
       <c r="A300" t="s" s="2">
-        <v>969</v>
+        <v>968</v>
       </c>
       <c r="B300" t="s" s="2">
         <v>724</v>
@@ -43860,7 +43859,7 @@
     </row>
     <row r="301" hidden="true">
       <c r="A301" t="s" s="2">
-        <v>970</v>
+        <v>969</v>
       </c>
       <c r="B301" t="s" s="2">
         <v>725</v>
@@ -43997,7 +43996,7 @@
     </row>
     <row r="302" hidden="true">
       <c r="A302" t="s" s="2">
-        <v>971</v>
+        <v>970</v>
       </c>
       <c r="B302" t="s" s="2">
         <v>730</v>
@@ -44132,7 +44131,7 @@
     </row>
     <row r="303" hidden="true">
       <c r="A303" t="s" s="2">
-        <v>972</v>
+        <v>971</v>
       </c>
       <c r="B303" t="s" s="2">
         <v>736</v>
@@ -44265,7 +44264,7 @@
     </row>
     <row r="304" hidden="true">
       <c r="A304" t="s" s="2">
-        <v>973</v>
+        <v>972</v>
       </c>
       <c r="B304" t="s" s="2">
         <v>805</v>
@@ -44398,7 +44397,7 @@
     </row>
     <row r="305" hidden="true">
       <c r="A305" t="s" s="2">
-        <v>974</v>
+        <v>973</v>
       </c>
       <c r="B305" t="s" s="2">
         <v>807</v>
@@ -44533,7 +44532,7 @@
     </row>
     <row r="306" hidden="true">
       <c r="A306" t="s" s="2">
-        <v>975</v>
+        <v>974</v>
       </c>
       <c r="B306" t="s" s="2">
         <v>809</v>
@@ -44668,7 +44667,7 @@
     </row>
     <row r="307" hidden="true">
       <c r="A307" t="s" s="2">
-        <v>976</v>
+        <v>975</v>
       </c>
       <c r="B307" t="s" s="2">
         <v>809</v>
@@ -44737,7 +44736,7 @@
       </c>
       <c r="Y307" s="2"/>
       <c r="Z307" t="s" s="2">
-        <v>977</v>
+        <v>976</v>
       </c>
       <c r="AA307" t="s" s="2">
         <v>84</v>
@@ -44805,7 +44804,7 @@
     </row>
     <row r="308" hidden="true">
       <c r="A308" t="s" s="2">
-        <v>978</v>
+        <v>977</v>
       </c>
       <c r="B308" t="s" s="2">
         <v>809</v>
@@ -44874,7 +44873,7 @@
       </c>
       <c r="Y308" s="2"/>
       <c r="Z308" t="s" s="2">
-        <v>979</v>
+        <v>978</v>
       </c>
       <c r="AA308" t="s" s="2">
         <v>84</v>
@@ -44942,7 +44941,7 @@
     </row>
     <row r="309" hidden="true">
       <c r="A309" t="s" s="2">
-        <v>980</v>
+        <v>979</v>
       </c>
       <c r="B309" t="s" s="2">
         <v>824</v>
@@ -45079,7 +45078,7 @@
     </row>
     <row r="310" hidden="true">
       <c r="A310" t="s" s="2">
-        <v>981</v>
+        <v>980</v>
       </c>
       <c r="B310" t="s" s="2">
         <v>743</v>
@@ -45214,7 +45213,7 @@
     </row>
     <row r="311" hidden="true">
       <c r="A311" t="s" s="2">
-        <v>982</v>
+        <v>981</v>
       </c>
       <c r="B311" t="s" s="2">
         <v>749</v>
@@ -45347,13 +45346,13 @@
     </row>
     <row r="312" hidden="true">
       <c r="A312" t="s" s="2">
-        <v>983</v>
+        <v>982</v>
       </c>
       <c r="B312" t="s" s="2">
         <v>715</v>
       </c>
       <c r="C312" t="s" s="2">
-        <v>984</v>
+        <v>983</v>
       </c>
       <c r="D312" t="s" s="2">
         <v>84</v>
@@ -45378,7 +45377,7 @@
         <v>716</v>
       </c>
       <c r="L312" t="s" s="2">
-        <v>985</v>
+        <v>984</v>
       </c>
       <c r="M312" t="s" s="2">
         <v>718</v>
@@ -45482,7 +45481,7 @@
     </row>
     <row r="313" hidden="true">
       <c r="A313" t="s" s="2">
-        <v>986</v>
+        <v>985</v>
       </c>
       <c r="B313" t="s" s="2">
         <v>723</v>
@@ -45615,7 +45614,7 @@
     </row>
     <row r="314" hidden="true">
       <c r="A314" t="s" s="2">
-        <v>987</v>
+        <v>986</v>
       </c>
       <c r="B314" t="s" s="2">
         <v>724</v>
@@ -45750,7 +45749,7 @@
     </row>
     <row r="315" hidden="true">
       <c r="A315" t="s" s="2">
-        <v>988</v>
+        <v>987</v>
       </c>
       <c r="B315" t="s" s="2">
         <v>725</v>
@@ -45887,7 +45886,7 @@
     </row>
     <row r="316" hidden="true">
       <c r="A316" t="s" s="2">
-        <v>989</v>
+        <v>988</v>
       </c>
       <c r="B316" t="s" s="2">
         <v>730</v>
@@ -46022,7 +46021,7 @@
     </row>
     <row r="317" hidden="true">
       <c r="A317" t="s" s="2">
-        <v>990</v>
+        <v>989</v>
       </c>
       <c r="B317" t="s" s="2">
         <v>736</v>
@@ -46155,7 +46154,7 @@
     </row>
     <row r="318" hidden="true">
       <c r="A318" t="s" s="2">
-        <v>991</v>
+        <v>990</v>
       </c>
       <c r="B318" t="s" s="2">
         <v>805</v>
@@ -46288,7 +46287,7 @@
     </row>
     <row r="319" hidden="true">
       <c r="A319" t="s" s="2">
-        <v>992</v>
+        <v>991</v>
       </c>
       <c r="B319" t="s" s="2">
         <v>807</v>
@@ -46423,7 +46422,7 @@
     </row>
     <row r="320" hidden="true">
       <c r="A320" t="s" s="2">
-        <v>993</v>
+        <v>992</v>
       </c>
       <c r="B320" t="s" s="2">
         <v>809</v>
@@ -46490,7 +46489,7 @@
       </c>
       <c r="Y320" s="2"/>
       <c r="Z320" t="s" s="2">
-        <v>994</v>
+        <v>993</v>
       </c>
       <c r="AA320" t="s" s="2">
         <v>84</v>
@@ -46558,7 +46557,7 @@
     </row>
     <row r="321" hidden="true">
       <c r="A321" t="s" s="2">
-        <v>995</v>
+        <v>994</v>
       </c>
       <c r="B321" t="s" s="2">
         <v>824</v>
@@ -46695,7 +46694,7 @@
     </row>
     <row r="322" hidden="true">
       <c r="A322" t="s" s="2">
-        <v>996</v>
+        <v>995</v>
       </c>
       <c r="B322" t="s" s="2">
         <v>743</v>
@@ -46830,7 +46829,7 @@
     </row>
     <row r="323" hidden="true">
       <c r="A323" t="s" s="2">
-        <v>997</v>
+        <v>996</v>
       </c>
       <c r="B323" t="s" s="2">
         <v>749</v>
@@ -46963,10 +46962,10 @@
     </row>
     <row r="324" hidden="true">
       <c r="A324" t="s" s="2">
-        <v>998</v>
+        <v>997</v>
       </c>
       <c r="B324" t="s" s="2">
-        <v>998</v>
+        <v>997</v>
       </c>
       <c r="C324" s="2"/>
       <c r="D324" t="s" s="2">
@@ -46989,19 +46988,19 @@
         <v>84</v>
       </c>
       <c r="K324" t="s" s="2">
+        <v>998</v>
+      </c>
+      <c r="L324" t="s" s="2">
         <v>999</v>
       </c>
-      <c r="L324" t="s" s="2">
+      <c r="M324" t="s" s="2">
         <v>1000</v>
       </c>
-      <c r="M324" t="s" s="2">
+      <c r="N324" t="s" s="2">
         <v>1001</v>
       </c>
-      <c r="N324" t="s" s="2">
+      <c r="O324" t="s" s="2">
         <v>1002</v>
-      </c>
-      <c r="O324" t="s" s="2">
-        <v>1003</v>
       </c>
       <c r="P324" t="s" s="2">
         <v>84</v>
@@ -47030,7 +47029,7 @@
       </c>
       <c r="Y324" s="2"/>
       <c r="Z324" t="s" s="2">
-        <v>1004</v>
+        <v>1003</v>
       </c>
       <c r="AA324" t="s" s="2">
         <v>84</v>
@@ -47048,7 +47047,7 @@
         <v>84</v>
       </c>
       <c r="AF324" t="s" s="2">
-        <v>998</v>
+        <v>997</v>
       </c>
       <c r="AG324" t="s" s="2">
         <v>85</v>
@@ -47084,13 +47083,13 @@
         <v>84</v>
       </c>
       <c r="AR324" t="s" s="2">
+        <v>1004</v>
+      </c>
+      <c r="AS324" t="s" s="2">
         <v>1005</v>
       </c>
-      <c r="AS324" t="s" s="2">
+      <c r="AT324" t="s" s="2">
         <v>1006</v>
-      </c>
-      <c r="AT324" t="s" s="2">
-        <v>1007</v>
       </c>
       <c r="AU324" t="s" s="2">
         <v>84</v>

</xml_diff>